<commit_message>
Salvare Codex: 2026-10-08T14:13:28.280906+00:00 (6 proiecte)
</commit_message>
<xml_diff>
--- a/Comun/Analizează și consolidează parolele din fișier Excel/fisiere/PIN-semnaturi electronice--cd708140.xlsx
+++ b/Comun/Analizează și consolidează parolele din fișier Excel/fisiere/PIN-semnaturi electronice--cd708140.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\parole\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D7CF6B4-0BBE-4392-A444-49436227DAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D866976A-97D5-4C3E-9DC0-75F02EE38966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27444" yWindow="2472" windowWidth="10032" windowHeight="12120" xr2:uid="{B652EA53-5765-4EF9-AC45-F958975AB6DF}"/>
+    <workbookView xWindow="28344" yWindow="3348" windowWidth="10032" windowHeight="12120" xr2:uid="{B652EA53-5765-4EF9-AC45-F958975AB6DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Semnatura</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>Coloană1</t>
+  </si>
+  <si>
+    <t>Florin Neamtiu</t>
   </si>
 </sst>
 </file>
@@ -159,8 +162,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2B87970B-60D1-472F-9837-125C51572347}" name="Table1" displayName="Table1" ref="A1:D8" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
-  <autoFilter ref="A1:D8" xr:uid="{2B87970B-60D1-472F-9837-125C51572347}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2B87970B-60D1-472F-9837-125C51572347}" name="Table1" displayName="Table1" ref="A1:D9" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A1:D9" xr:uid="{2B87970B-60D1-472F-9837-125C51572347}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{2C399471-5F94-45C9-8C44-3057D7A78438}" name="Semnatura" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{7EB0ED10-1339-409E-B763-57AECCB97926}" name="PIN" dataDxfId="2"/>
@@ -468,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46E35A1C-FFD8-4DDD-830F-8FB3D130585A}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.44140625" customWidth="1"/>
@@ -573,6 +576,16 @@
         <v>13</v>
       </c>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="1">
+        <v>34347047</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>